<commit_message>
update on oct 19
</commit_message>
<xml_diff>
--- a/12600895.xlsx
+++ b/12600895.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ba3379cbd202792/Desktop/PYTHON/776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{8224F70C-BBF1-4898-9E15-74A4031B271A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E46DDF8C-C3CA-4108-93D1-AD8931DCC1C0}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{8224F70C-BBF1-4898-9E15-74A4031B271A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1F4A314-27C6-46E0-BF08-7EC8265B13D9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -223,6 +223,15 @@
   </si>
   <si>
     <t>MSc IT/ D1P2648</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hectic schedule </t>
   </si>
 </sst>
 </file>
@@ -503,6 +512,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1140,26 +1153,50 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="A9" s="13">
+        <v>46313</v>
+      </c>
+      <c r="B9" s="14">
+        <v>420</v>
+      </c>
+      <c r="C9" s="14">
+        <v>45</v>
+      </c>
+      <c r="D9" s="14">
+        <v>155</v>
+      </c>
+      <c r="E9" s="14">
+        <v>55</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0</v>
+      </c>
+      <c r="G9" s="14">
+        <v>0</v>
+      </c>
+      <c r="H9" s="14">
+        <v>110</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>785</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>655</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>

</xml_diff>

<commit_message>
update on oct 20
</commit_message>
<xml_diff>
--- a/12600895.xlsx
+++ b/12600895.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ba3379cbd202792/Desktop/PYTHON/776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{8224F70C-BBF1-4898-9E15-74A4031B271A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1F4A314-27C6-46E0-BF08-7EC8265B13D9}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{8224F70C-BBF1-4898-9E15-74A4031B271A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51779079-6A5D-48D3-ADB8-AF78C3B50E18}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -199,15 +199,6 @@
   </si>
   <si>
     <t>5. GOOD PRACTICE</t>
-  </si>
-  <si>
-    <t>Excellent</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>day went well</t>
   </si>
   <si>
     <t>Neutral</t>
@@ -923,7 +914,7 @@
         <v>30</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
@@ -940,7 +931,7 @@
         <v>32</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C3" s="20"/>
       <c r="D3" s="20"/>
@@ -948,7 +939,7 @@
         <v>33</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G3" s="20"/>
     </row>
@@ -1061,54 +1052,24 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
-        <v>46288</v>
-      </c>
-      <c r="B7" s="14">
-        <v>450</v>
-      </c>
-      <c r="C7" s="14">
-        <v>40</v>
-      </c>
-      <c r="D7" s="14">
-        <v>70</v>
-      </c>
-      <c r="E7" s="14">
-        <v>50</v>
-      </c>
-      <c r="F7" s="14">
-        <v>300</v>
-      </c>
-      <c r="G7" s="14">
-        <v>6</v>
-      </c>
-      <c r="H7" s="14">
-        <v>20</v>
-      </c>
-      <c r="I7" s="15">
-        <f t="shared" si="0"/>
-        <v>930</v>
-      </c>
-      <c r="J7" s="15">
-        <f t="shared" si="1"/>
-        <v>510</v>
-      </c>
-      <c r="K7" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="L7" s="16" t="s">
-        <v>50</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="N7" s="17" t="s">
-        <v>56</v>
-      </c>
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="B8" s="14">
         <v>420</v>
@@ -1140,7 +1101,7 @@
         <v>580</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="L8" s="16" t="s">
         <v>50</v>
@@ -1149,12 +1110,12 @@
         <v>51</v>
       </c>
       <c r="N8" s="17" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="B9" s="14">
         <v>420</v>
@@ -1186,16 +1147,16 @@
         <v>655</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="L9" s="16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="N9" s="17" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -9831,21 +9792,21 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J401">
+  <conditionalFormatting sqref="J6 J8:J401">
     <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6:K401" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Please choose a value from the dropdown list." prompt="Select today's overall feeling" sqref="K6 K8:K401" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Excellent,Good,Neutral,Low,Stressed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6:L401" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's satisfaction level" sqref="L6 L8:L401" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Very Satisfied,Satisfied,Neutral,Unsatisfied,Very Unsatisfied"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6:M401" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" allowBlank="1" prompt="Select today's energy level" sqref="M6 M8:M401" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
update on oct 30
</commit_message>
<xml_diff>
--- a/12600895.xlsx
+++ b/12600895.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\PYTHON\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4094B2-3598-43C8-9DA7-5F2011341ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE7DEBD-8F84-4E82-8AE0-25E01B6BABA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>Today, I grew a little.</t>
+  </si>
+  <si>
+    <t>Every day is a new chance.</t>
   </si>
 </sst>
 </file>
@@ -1410,26 +1413,50 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="13">
+        <v>46325</v>
+      </c>
+      <c r="B15" s="14">
+        <v>420</v>
+      </c>
+      <c r="C15" s="14">
+        <v>45</v>
+      </c>
+      <c r="D15" s="14">
+        <v>180</v>
+      </c>
+      <c r="E15" s="14">
+        <v>65</v>
+      </c>
+      <c r="F15" s="14">
+        <v>250</v>
+      </c>
+      <c r="G15" s="14">
+        <v>5</v>
+      </c>
+      <c r="H15" s="14">
+        <v>80</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
+        <v>400</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>

</xml_diff>